<commit_message>
feat: pipeline de dados unificado e modelo relacional normalizado
</commit_message>
<xml_diff>
--- a/data/processed/arbitros.xlsx
+++ b/data/processed/arbitros.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,7 +449,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -469,7 +469,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -489,7 +489,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -509,7 +509,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -529,7 +529,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -849,7 +849,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -949,10 +949,30 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>REFEREE</t>
+          <t>Árbitro</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>75722</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Paulo Cesar Zanovelli da Silva</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Árbitro</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
         <is>
           <t>Brazil</t>
         </is>

</xml_diff>

<commit_message>
refactor: unifica pipeline silver, traduz posicoes faltantes e tipa datas em datetime
</commit_message>
<xml_diff>
--- a/data/processed/arbitros.xlsx
+++ b/data/processed/arbitros.xlsx
@@ -429,12 +429,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>tipo_arbitro</t>
+          <t>nacionalidade</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>nacionalidade</t>
+          <t>tipo</t>
         </is>
       </c>
     </row>
@@ -449,12 +449,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -469,12 +469,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -489,12 +489,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -529,12 +529,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -549,12 +549,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -589,12 +589,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -609,12 +609,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -649,12 +649,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -669,12 +669,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -709,12 +709,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -729,12 +729,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -769,12 +769,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -789,12 +789,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -829,12 +829,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -849,12 +849,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -869,12 +869,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -889,12 +889,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -909,12 +909,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -929,12 +929,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -949,12 +949,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>
@@ -969,12 +969,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Árbitro</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Árbitro</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: valida checklist final de entregaveis do projeto
</commit_message>
<xml_diff>
--- a/data/processed/arbitros.xlsx
+++ b/data/processed/arbitros.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -978,6 +978,26 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>60911</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Luiz Alexandre Fernandes</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Árbitro</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>